<commit_message>
Refine Chao2 analysis and update figures
Updated the scoring methods Rmd to estimate Chao2 on collapsed `monotonic_score_id` methods, add a consistency check against the reported collapsed score count, report Q1/Q2 and log-normal CIs, and include a raw `score_id` sensitivity analysis to preserve reproducibility of the previous estimate. Also corrected the clinical protocol cross-tab query, switched multiverse histogram colors to the new palette, and regenerated related plot and spreadsheet outputs.
</commit_message>
<xml_diff>
--- a/code/multiverse/most_frequent_scoring_strategies.xlsx
+++ b/code/multiverse/most_frequent_scoring_strategies.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -982,6 +982,198 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>4016</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>"amount of gained money"</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>12</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>money</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>money</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>indeterminable</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>01 to 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>1010</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>deck selections [(C+D)-(A+B)] for blocks 3, 4, and 5, within 5 blocks (last 60% of trials)</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>deck selections</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>net score</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>(C+D)-(A+B)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>41 to 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>1008</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>deck selections [(C+D)-(A+B)] for blocks 1 and 2, within 5 blocks (first 40% of trials)</t>
+        </is>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>deck selections</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>net score</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>(C+D)-(A+B)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>01 to 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>1066</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>deck selections (A+C) across all trials (100% of trials)</t>
+        </is>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>deck selections</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>loss frequency based score</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(A+C)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>01 to 100</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>